<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.001-04 Amir et le gâteau encore chaud
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.001-04.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.001-04.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, matin</t>
+          <t>cuisine, matin, gâteau, saladier, assiette, miette, carrelage, four, fenêtre, beurre, citron, table</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Le soleil chauffe le carrelage. Amir sent le gâteau. Il dit sa joie. Il partage deux petits bouts.</t>
+          <t>Maman pose le saladier près du gâteau. Sur le verre, un éclat de saladier luit. Amir veut un bout, maintenant. Le gâteau est trop chaud. Poitrine trop vite. Sourire parti. Papa s'accroupit. Un sourire revient. Je suis content. Merci vécu. Deux petits bouts. Deuxième ruse : le bout s'effrite. Il refuse de foncer. Un éclat de saladier tient sur le verre.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil pose des carrés chauds. Les carrés sont sur le carrelage. La cuisine sent le beurre. Un gâteau refroidit près de la fenêtre. Il est encore un peu chaud. Une mouche tapote le carreau. Papa essuie la table. La nappe a des petits pois. Maman range le saladier. Le saladier fait un bruit. Amir, tu sens le gâteau ? Oui, maman. C'est bon. Viens. On le regarde. En ce moment, Amir avance. Ses pieds touchent un carré de soleil. Le carrelage est chaud. Amir pose une main au mur. Le mur est lisse. Le gâteau est jaune et rond. Une miette est déjà tombée. Amir se penche tout près. Ça sent le citron. Tu veux une petite assiette ? Oui. Maman coupe deux petits bouts. Parce que le gâteau est là. Les joues d'Amir sont chaudes. Son ventre est léger. Un sourire arrive. Je suis content. C'est de la joie. Bravo, Amir. Tu as dit ta joie. On peut partager ? Oui. On partage. Amir prend un bout. Papa prend un bout. Ils goûtent ensemble. C'est doux. C'est un peu citron. Maman, un bout ? Merci, Amir. Tu m'invites. Je suis content. Tu as de la joie ? Oui, papa. Le soleil reste sur le sol. La nappe bouge un peu. Le gâteau sent encore bon.</t>
+          <t>Maman pose le saladier près du gâteau. Il est grand, maman. Tu le vois, le saladier ? Oui, maman. Sur le verre, un éclat de saladier luit. Il brille, papa. Le soleil le touche ? Oui, un petit point. Papa ouvre la fenêtre d'un cran. L'air arrive. Tu le sens, l'air ? Oui, maman. La cuisine sent le beurre. Ça sent le citron. Le citron, Amir ? Oui, papa. Le gâteau est jaune et rond. Il est beau ! Il est chaud, Amir ? Un peu, maman. Le carrelage tient la chaleur du four. Il est tiède, sous les pieds. Tes pieds sont au chaud ? Oui, papa. Une mouche tapote le carreau. Toc, maman. Tu l'entends, Amir ? Oui, maman. Une miette glisse du bord. Une miette ! Tu la vois, Amir ? Oui, sur la table. Maman pose une petite assiette. Pour le bout ? Elle attend, Amir. Un carré de soleil pose sur le carrelage. Il est chaud, le carré. Tu le touches, Amir ? Oui, papa. Amir se penche tout près. Ça chauffe le nez. Tu le sens, le gâteau ? Oui, il fume. Une petite fumée monte. Je veux un bout, maintenant ! Tout de suite ? Oui, papa. En ce moment, Amir tend la main. Ses doigts touchent le gâteau. Le gâteau est trop chaud. Aïe ! Amir retire la main, trop vite. Le sourire d'Amir disparaît. Sa poitrine va trop vite. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le gâteau, Amir ? Oui, papa. Tes doigts sont chauds, Amir ? Un peu, maman. L'éclat de saladier tremble, puis tient. Les joues d'Amir redeviennent chaudes. Son ventre est léger. Un sourire revient, tout petit.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil pose des carrés chauds. Les carrés sont sur le carrelage. La cuisine sent le beurre. Un gâteau refroidit près de la fenêtre. Il est encore un peu chaud. Une mouche tapote le carreau. Papa essuie la table. La nappe a des petits pois. Maman range le saladier. Le saladier fait un bruit. Amir, tu sens le gâteau ? Oui, maman. C'est bon. Viens. On le regarde. En ce moment, Amir avance. Ses pieds touchent un carré de soleil. Le carrelage est chaud. Amir pose une main au mur. Le mur est lisse. Le gâteau est jaune et rond. Une miette est déjà tombée. Amir se penche tout près. Ça sent le citron. Tu veux une petite assiette ? Oui. Maman coupe deux petits bouts. Parce que le gâteau est là. Les joues d'Amir sont chaudes. Son ventre est léger. Un sourire arrive. Je suis content. C'est de la joie. Bravo, Amir. Tu as dit ta joie. On peut partager ? Oui. On partage. Amir prend un bout. Papa prend un bout. Ils goûtent ensemble. C'est doux. C'est un peu citron. Maman, un bout ? Merci, Amir. Tu m'invites. Je suis content. Tu as de la joie ? Oui, papa. Le soleil reste sur le sol. La nappe bouge un peu. Le gâteau sent encore bon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pose le saladier près du gâteau. Il est grand, maman. Tu le vois, le saladier ? Oui, maman. Sur le verre, un &lt;emphasis level="moderate"&gt;éclat de saladier&lt;/emphasis&gt; luit. Il brille, papa. Le soleil le touche ? Oui, un petit point. Papa ouvre la fenêtre d'un cran. L'air arrive. Tu le sens, l'air ? Oui, maman. La cuisine sent le beurre. Ça sent le citron. Le citron, Amir ? Oui, papa. Le gâteau est jaune et rond. Il est beau ! Il est chaud, Amir ? Un peu, maman. Le carrelage tient la chaleur du four. Il est tiède, sous les pieds. Tes pieds sont au chaud ? Oui, papa. Une mouche tapote le carreau. Toc, maman. Tu l'entends, Amir ? Oui, maman. Une miette glisse du bord. Une miette ! Tu la vois, Amir ? Oui, sur la table. Maman pose une petite assiette. Pour le bout ? Elle attend, Amir. Un carré de soleil pose sur le carrelage. Il est chaud, le carré. Tu le touches, Amir ? Oui, papa. Amir se penche tout près. Ça chauffe le nez. Tu le sens, le gâteau ? Oui, il fume. Une petite fumée monte. Je veux un bout, maintenant ! Tout de suite ? Oui, papa. En ce moment, Amir tend la main. Ses doigts touchent le gâteau. Le gâteau est trop chaud. Aïe ! Amir retire la main, trop vite. Le sourire d'Amir disparaît. Sa poitrine va trop vite. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le gâteau, Amir ? Oui, papa. Tes doigts sont chauds, Amir ? Un peu, maman. L'éclat de saladier tremble, puis tient. Les joues d'Amir redeviennent chaudes. Son ventre est léger. Un sourire revient, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Flora entre dans la cuisine. Maman est là. Ça sent le gâteau. Le gâteau est encore chaud. Flora sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Flora dit : je suis &lt;emphasis&gt;content&lt;/emphasis&gt;e. Maman dit : c'est de la joie. Flora prend une petite assiette. Elle dit : on peut partager. Maman coupe deux petits bouts. Flora prend un bout. Maman prend un bout. Ils goûtent ensemble. C'est doux. C'est un peu vanillé. Flora dit encore : je suis contente. La joie est là, dans la cuisine. Maman sourit. Partager, c'est bien. Flora essuie ses doigts. Le gâteau sent encore bon.&lt;/slow&gt; [pause]</t>
+          <t>Maman pose le saladier près du gâteau. Il est grand, maman. Tu le vois, le saladier ? Oui, maman. Sur le verre, un &lt;emphasis&gt;éclat de saladier&lt;/emphasis&gt; luit. Il brille, papa. Le soleil le touche ? Oui, un petit point. Papa ouvre la fenêtre d'un cran. L'air arrive. Tu le sens, l'air ? Oui, maman. La cuisine sent le beurre. Ça sent le citron. Le citron, Amir ? Oui, papa. Le gâteau est jaune et rond. Il est beau ! Il est chaud, Amir ? Un peu, maman. Le carrelage tient la chaleur du four. Il est tiède, sous les pieds. Tes pieds sont au chaud ? Oui, papa. Une mouche tapote le carreau. Toc, maman. Tu l'entends, Amir ? Oui, maman. Une miette glisse du bord. Une miette ! Tu la vois, Amir ? Oui, sur la table. Maman pose une petite assiette. Pour le bout ? Elle attend, Amir. Un carré de soleil pose sur le carrelage. Il est chaud, le carré. Tu le touches, Amir ? Oui, papa. Amir se penche tout près. Ça chauffe le nez. Tu le sens, le gâteau ? Oui, il fume. Une petite fumée monte. Je veux un bout, maintenant ! Tout de suite ? Oui, papa. En ce moment, Amir tend la main. Ses doigts touchent le gâteau. Le gâteau est trop chaud. Aïe ! Amir retire la main, trop vite. Le sourire d'Amir disparaît. Sa poitrine va trop vite. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le gâteau, Amir ? Oui, papa. Tes doigts sont chauds, Amir ? Un peu, maman. L'éclat de saladier tremble, puis tient. Les joues d'Amir redeviennent chaudes. Son ventre est léger. Un sourire revient, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>éclat de saladier</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,59 +1319,81 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_un_bout_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le soleil pose des carrés chauds.
-narrateur|Les carrés sont sur le carrelage.
+          <t>narrateur|Maman pose le saladier près du gâteau.
+enfant-m|Il est grand, maman.
+maman|Tu le vois, le saladier ?
+enfant-m|Oui, maman.
+narrateur|Sur le verre, un éclat de saladier luit.
+enfant-m|Il brille, papa.
+papa|Le soleil le touche ?
+enfant-m|Oui, un petit point.
+narrateur|Papa ouvre la fenêtre d'un cran.
+enfant-m|L'air arrive.
+maman|Tu le sens, l'air ?
+enfant-m|Oui, maman.
 narrateur|La cuisine sent le beurre.
-narrateur|Un gâteau refroidit près de la fenêtre.
-narrateur|Il est encore un peu chaud.
+enfant-m|Ça sent le citron.
+papa|Le citron, Amir ?
+enfant-m|Oui, papa.
+narrateur|Le gâteau est jaune et rond.
+enfant-m|Il est beau !
+maman|Il est chaud, Amir ?
+enfant-m|Un peu, maman.
+narrateur|Le carrelage tient la chaleur du four.
+enfant-m|Il est tiède, sous les pieds.
+papa|Tes pieds sont au chaud ?
+enfant-m|Oui, papa.
 narrateur|Une mouche tapote le carreau.
-narrateur|Papa essuie la table.
-narrateur|La nappe a des petits pois.
-narrateur|Maman range le saladier.
-narrateur|Le saladier fait un bruit.
-maman|Amir, tu sens le gâteau ?
-enfant-m|Oui, maman. C'est bon.
-papa|Viens. On le regarde.
-narrateur|En ce moment, Amir avance.
-narrateur|Ses pieds touchent un carré de soleil.
-narrateur|Le carrelage est chaud.
-narrateur|Amir pose une main au mur.
-narrateur|Le mur est lisse.
-narrateur|Le gâteau est jaune et rond.
-narrateur|Une miette est déjà tombée.
+enfant-m|Toc, maman.
+maman|Tu l'entends, Amir ?
+enfant-m|Oui, maman.
+narrateur|Une miette glisse du bord.
+enfant-m|Une miette !
+maman|Tu la vois, Amir ?
+enfant-m|Oui, sur la table.
+narrateur|Maman pose une petite assiette.
+enfant-m|Pour le bout ?
+maman|Elle attend, Amir.
+narrateur|Un carré de soleil pose sur le carrelage.
+enfant-m|Il est chaud, le carré.
+papa|Tu le touches, Amir ?
+enfant-m|Oui, papa.
 narrateur|Amir se penche tout près.
-narrateur|Ça sent le citron.
-maman|Tu veux une petite assiette ?
-enfant-m|Oui.
-narrateur|Maman coupe deux petits bouts.
-narrateur|Parce que le gâteau est là.
-narrateur|Les joues d'Amir sont chaudes.
+enfant-m|Ça chauffe le nez.
+papa|Tu le sens, le gâteau ?
+enfant-m|Oui, il fume.
+narrateur|Une petite fumée monte.
+enfant-m|Je veux un bout, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|En ce moment, Amir tend la main.
+narrateur|Ses doigts touchent le gâteau.
+narrateur|Le gâteau est trop chaud.
+enfant-m|Aïe !
+narrateur|Amir retire la main, trop vite.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Sa poitrine va trop vite.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois le gâteau, Amir ?
+enfant-m|Oui, papa.
+maman|Tes doigts sont chauds, Amir ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de saladier tremble, puis tient.
+narrateur|Les joues d'Amir redeviennent chaudes.
 narrateur|Son ventre est léger.
-narrateur|Un sourire arrive.
-enfant-m|Je suis content.
-maman|C'est de la joie.
-papa|Bravo, Amir.
-papa|Tu as dit ta joie.
-enfant-m|On peut partager ?
-papa|Oui. On partage.
-narrateur|Amir prend un bout.
-narrateur|Papa prend un bout.
-narrateur|Ils goûtent ensemble.
-narrateur|C'est doux. C'est un peu citron.
-enfant-m|Maman, un bout ?
-maman|Merci, Amir.
-maman|Tu m'invites.
-enfant-m|Je suis content.
-papa|Tu as de la joie ?
-enfant-m|Oui, papa.
-narrateur|Le soleil reste sur le sol.
-narrateur|La nappe bouge un peu.
-narrateur|Le gâteau sent encore bon.</t>
+narrateur|Un sourire revient, tout petit.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1408,12 +1430,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir sourit. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Amir&lt;/emphasis&gt; sourit. Que dit-il ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Flora sourit. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Amir&lt;/emphasis&gt; sourit. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1438,7 +1460,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Flora sent de la joie. Que dit-elle ?</t>
+          <t>Amir sent de la joie. Que dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1476,7 +1498,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1487,7 +1509,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1502,34 +1524,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Amir</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1544,7 +1570,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1554,12 +1580,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=amir_sourit_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Amir sourit. Que dit-il ?</t>
+          <t>narrateur|Amir sourit.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1613,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir mâche son petit bout. C'est de la joie. Oui. Tu es content. Tu as partagé. Tu as fini ton bout ? Oui. Amir essuie ses doigts. L'assiette est presque vide. Une miette reste au bord. Tu as du citron sur les lèvres. C'est doux.</t>
+          <t>Amir veut un bout, tout de suite. Je prends, maintenant ! Sa main avance, trop vite. Puis il s'arrête. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le gâteau, un instant. Il écoute la cuisine. Je suis content. Le gâteau est là, Amir ? Oui, papa. On peut partager ? On coupe deux petits bouts ? Oui, deux. Maman prend la petite assiette. Elle coupe un bout, sans se presser. Tu attends, Amir ? Oui, papa. Le bout pose une miette. Une miette, maman. Elle reste sur l'assiette ? Oui, maman. Amir prend le bout, sans se presser. Papa, un bout ? Merci, Amir. Papa reste à la même hauteur. Ils goûtent ensemble, tout près. C'est un peu citron. C'est doux, Amir ? Oui, papa. Le citron est sur les lèvres, Amir ? C'est doux. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près du gâteau ? Oui. L'assiette est tiède, Amir ? Un peu, maman. Le gâteau attend sur la table. Il a un trou. Tu le vois, le trou ? Oui, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir mâche son petit bout. C'est de la joie. Oui. Tu es content. Tu as partagé. Tu as fini ton bout ? Oui. Amir essuie ses doigts. L'assiette est presque vide. Une miette reste au bord. Tu as du citron sur les lèvres. C'est doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut un bout, tout de suite. Je prends, maintenant ! Sa main avance, trop vite. Puis il s'arrête. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le gâteau, un instant. Il écoute la cuisine. Je suis &lt;emphasis level="moderate"&gt;content&lt;/emphasis&gt;. Le gâteau est là, Amir ? Oui, papa. On peut partager ? On coupe deux petits bouts ? Oui, deux. Maman prend la petite assiette. Elle coupe un bout, sans se presser. Tu attends, Amir ? Oui, papa. Le bout pose une miette. Une miette, maman. Elle reste sur l'assiette ? Oui, maman. Amir prend le bout, sans se presser. Papa, un bout ? Merci, Amir. Papa reste à la même hauteur. Ils goûtent ensemble, tout près. C'est un peu citron. C'est doux, Amir ? Oui, papa. Le citron est sur les lèvres, Amir ? C'est doux. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près du gâteau ? Oui. L'assiette est tiède, Amir ? Un peu, maman. Le gâteau attend sur la table. Il a un trou. Tu le vois, le trou ? Oui, papa.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Flora a nommé sa joie. Elle a partagé avec maman. Être &lt;emphasis&gt;content&lt;/emphasis&gt;, c'est bien.&lt;/slow&gt; [pause]</t>
+          <t>Amir veut un bout, tout de suite. Je prends, maintenant ! Sa main avance, trop vite. Puis il s'arrête. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le gâteau, un instant. Il écoute la cuisine. Je suis &lt;emphasis&gt;content&lt;/emphasis&gt;. Le gâteau est là, Amir ? Oui, papa. On peut partager ? On coupe deux petits bouts ? Oui, deux. Maman prend la petite assiette. Elle coupe un bout, sans se presser. Tu attends, Amir ? Oui, papa. Le bout pose une miette. Une miette, maman. Elle reste sur l'assiette ? Oui, maman. Amir prend le bout, sans se presser. Papa, un bout ? Merci, Amir. Papa reste à la même hauteur. Ils goûtent ensemble, tout près. C'est un peu citron. C'est doux, Amir ? Oui, papa. Le citron est sur les lèvres, Amir ? C'est doux. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près du gâteau ? Oui. L'assiette est tiède, Amir ? Un peu, maman. Le gâteau attend sur la table. Il a un trou. Tu le vois, le trou ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,18 +1670,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1684,23 +1711,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1736,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,26 +1748,58 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_dit_content_il_partage; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir mâche son petit bout.
-enfant-m|C'est de la joie.
-maman|Oui. Tu es content.
-maman|Tu as partagé.
-papa|Tu as fini ton bout ?
+          <t>narrateur|Amir veut un bout, tout de suite.
+enfant-m|Je prends, maintenant !
+narrateur|Sa main avance, trop vite.
+narrateur|Puis il s'arrête.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le gâteau, un instant.
+narrateur|Il écoute la cuisine.
+enfant-m|Je suis content.
+papa|Le gâteau est là, Amir ?
+enfant-m|Oui, papa.
+enfant-m|On peut partager ?
+maman|On coupe deux petits bouts ?
+enfant-m|Oui, deux.
+narrateur|Maman prend la petite assiette.
+narrateur|Elle coupe un bout, sans se presser.
+papa|Tu attends, Amir ?
+enfant-m|Oui, papa.
+narrateur|Le bout pose une miette.
+enfant-m|Une miette, maman.
+maman|Elle reste sur l'assiette ?
+enfant-m|Oui, maman.
+narrateur|Amir prend le bout, sans se presser.
+enfant-m|Papa, un bout ?
+papa|Merci, Amir.
+narrateur|Papa reste à la même hauteur.
+narrateur|Ils goûtent ensemble, tout près.
+enfant-m|C'est un peu citron.
+papa|C'est doux, Amir ?
+enfant-m|Oui, papa.
+maman|Le citron est sur les lèvres, Amir ?
+enfant-m|C'est doux.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du gâteau ?
 enfant-m|Oui.
-narrateur|Amir essuie ses doigts.
-narrateur|L'assiette est presque vide.
-narrateur|Une miette reste au bord.
-maman|Tu as du citron sur les lèvres.
-enfant-m|C'est doux.</t>
+maman|L'assiette est tiède, Amir ?
+enfant-m|Un peu, maman.
+narrateur|Le gâteau attend sur la table.
+enfant-m|Il a un trou.
+papa|Tu le vois, le trou ?
+enfant-m|Oui, papa.</t>
         </is>
       </c>
     </row>
@@ -1767,17 +1826,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Amir pose l'assiette. La cuisine est calme. Une miette reste sur la table. Tu veux un peu d'eau ? Une gorgée. Amir boit une gorgée. On reste un peu ? Oui, maman. Tu as bien invité. Je suis content. La joie est là. Le soleil touche encore le gâteau. Ils restent près de la table.</t>
+          <t>Maman pousse l'assiette près du gâteau. Elle est un peu collante. L'autre bout, maintenant ! Maman coupe le deuxième bout. Le bout s'effrite sur l'assiette. Il tombe ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le gâteau, un instant. Il écoute la cuisine, près de la table. Sur le verre, un éclat de saladier luit. Là, sur le saladier. On tient le bout ? Oui, papa. Le bout sent le beurre chaud. Une miette reste au bord. Amir pose le bout, sans se presser. Pour maman. Le gâteau est tiède, Amir ? Un peu. Maman prend le petit bout. L'assiette est calme, Amir ? Oui, papa. Un rayon passe sur le verre. Il allume le point. Tu vois le point, Amir ? Oui, papa. Deux petits bouts restent entre eux. On a partagé. Le gâteau a un trou, Amir ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le saladier reste près du gâteau. Il sent le beurre. On reste ici, Amir ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Amir pose l'assiette. La cuisine est calme. Une miette reste sur la table. Tu veux un peu d'eau ? Une gorgée. Amir boit une gorgée. On reste un peu ? Oui, maman. Tu as bien invité. Je suis content. La joie est là. Le soleil touche encore le gâteau. Ils restent près de la table.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pousse l'assiette près du gâteau. Elle est un peu collante. L'autre bout, maintenant ! Maman coupe le deuxième bout. Le bout s'effrite sur l'assiette. Il tombe ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le gâteau, un instant. Il écoute la cuisine, près de la table. Sur le verre, un &lt;emphasis level="moderate"&gt;éclat de saladier&lt;/emphasis&gt; luit. Là, sur le saladier. On tient le bout ? Oui, papa. Le bout sent le beurre chaud. Une miette reste au bord. Amir pose le bout, sans se presser. Pour maman. Le gâteau est tiède, Amir ? Un peu. Maman prend le petit bout. L'assiette est calme, Amir ? Oui, papa. Un rayon passe sur le verre. Il allume le point. Tu vois le point, Amir ? Oui, papa. Deux petits bouts restent entre eux. On a partagé. Le gâteau a un trou, Amir ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le saladier reste près du gâteau. Il sent le beurre. On reste ici, Amir ? Oui.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Flora range l'assiette. Maman lui prend la &lt;emphasis&gt;main&lt;/emphasis&gt;.&lt;/slow&gt; [pause]</t>
+          <t>Maman pousse l'assiette près du gâteau. Elle est un peu collante. L'autre bout, maintenant ! Maman coupe le deuxième bout. Le bout s'effrite sur l'assiette. Il tombe ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le gâteau, un instant. Il écoute la cuisine, près de la table. Sur le verre, un &lt;emphasis&gt;éclat de saladier&lt;/emphasis&gt; luit. Là, sur le saladier. On tient le bout ? Oui, papa. Le bout sent le beurre chaud. Une miette reste au bord. Amir pose le bout, sans se presser. Pour maman. Le gâteau est tiède, Amir ? Un peu. Maman prend le petit bout. L'assiette est calme, Amir ? Oui, papa. Un rayon passe sur le verre. Il allume le point. Tu vois le point, Amir ? Oui, papa. Deux petits bouts restent entre eux. On a partagé. Le gâteau a un trou, Amir ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le saladier reste près du gâteau. Il sent le beurre. On reste ici, Amir ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1824,18 +1883,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1858,30 +1917,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de saladier</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1890,10 +1949,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1902,24 +1961,55 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_bout_s_effrite_il_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose l'assiette.
-narrateur|La cuisine est calme.
-narrateur|Une miette reste sur la table.
-maman|Tu veux un peu d'eau ?
-enfant-m|Une gorgée.
-narrateur|Amir boit une gorgée.
-maman|On reste un peu ?
-enfant-m|Oui, maman.
-papa|Tu as bien invité.
-enfant-m|Je suis content.
-maman|La joie est là.
-narrateur|Le soleil touche encore le gâteau.
-narrateur|Ils restent près de la table.</t>
+          <t>narrateur|Maman pousse l'assiette près du gâteau.
+narrateur|Elle est un peu collante.
+enfant-m|L'autre bout, maintenant !
+narrateur|Maman coupe le deuxième bout.
+narrateur|Le bout s'effrite sur l'assiette.
+enfant-m|Il tombe !
+narrateur|Amir avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Amir refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le gâteau, un instant.
+narrateur|Il écoute la cuisine, près de la table.
+narrateur|Sur le verre, un éclat de saladier luit.
+enfant-m|Là, sur le saladier.
+papa|On tient le bout ?
+enfant-m|Oui, papa.
+narrateur|Le bout sent le beurre chaud.
+narrateur|Une miette reste au bord.
+narrateur|Amir pose le bout, sans se presser.
+enfant-m|Pour maman.
+maman|Le gâteau est tiède, Amir ?
+enfant-m|Un peu.
+narrateur|Maman prend le petit bout.
+papa|L'assiette est calme, Amir ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur le verre.
+enfant-m|Il allume le point.
+papa|Tu vois le point, Amir ?
+enfant-m|Oui, papa.
+narrateur|Deux petits bouts restent entre eux.
+enfant-m|On a partagé.
+papa|Le gâteau a un trou, Amir ?
+enfant-m|Oui, papa.
+maman|Tes genoux sont au chaud ?
+enfant-m|Un peu, maman.
+narrateur|Le saladier reste près du gâteau.
+enfant-m|Il sent le beurre.
+papa|On reste ici, Amir ?
+enfant-m|Oui.</t>
         </is>
       </c>
     </row>
@@ -1946,17 +2036,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis content. On a partagé. Bravo, Amir.</t>
+          <t>Ils restent près de la table. Maman essuie une miette. Le gâteau était trop chaud, papa. Tu l'as senti, toi ? Oui, près des doigts. On est bien, ici. Amir tapote le verre du saladier. Il a une trace de beurre. Tu la vois, la trace ? Oui, maman. Le gâteau est resté, Amir. Oui, avec le trou. Ça sent le citron, un peu tiède. Et le beurre, maman. Oui, dans l'air. La cuisine est calme, Amir ? Oui, papa. Deux petits bouts ont suffi. Un éclat de saladier tient sur le verre.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis content. On a partagé. Bravo, Amir.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman essuie une miette. Le gâteau était trop chaud, papa. Tu l'as senti, toi ? Oui, près des doigts. On est bien, ici. Amir tapote le verre du saladier. Il a une trace de beurre. Tu la vois, la trace ? Oui, maman. Le gâteau est resté, Amir. Oui, avec le trou. Ça sent le citron, un peu tiède. Et le beurre, maman. Oui, dans l'air. La cuisine est calme, Amir ? Oui, papa. Deux petits bouts ont suffi. Un &lt;emphasis level="moderate"&gt;éclat de saladier&lt;/emphasis&gt; tient sur le verre.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman essuie une miette. Le gâteau était trop chaud, papa. Tu l'as senti, toi ? Oui, près des doigts. On est bien, ici. Amir tapote le verre du saladier. Il a une trace de beurre. Tu la vois, la trace ? Oui, maman. Le gâteau est resté, Amir. Oui, avec le trou. Ça sent le citron, un peu tiède. Et le beurre, maman. Oui, dans l'air. La cuisine est calme, Amir ? Oui, papa. Deux petits bouts ont suffi. Un &lt;emphasis&gt;éclat de saladier&lt;/emphasis&gt; tient sur le verre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2003,7 +2093,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2011,7 +2101,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2023,12 +2113,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2037,14 +2127,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de saladier</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2056,11 +2150,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2069,26 +2163,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_verre; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis content.
-enfant-m|On a partagé.
-papa|Bravo, Amir.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman essuie une miette.
+enfant-m|Le gâteau était trop chaud, papa.
+papa|Tu l'as senti, toi ?
+enfant-m|Oui, près des doigts.
+maman|On est bien, ici.
+narrateur|Amir tapote le verre du saladier.
+enfant-m|Il a une trace de beurre.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le gâteau est resté, Amir.
+enfant-m|Oui, avec le trou.
+narrateur|Ça sent le citron, un peu tiède.
+enfant-m|Et le beurre, maman.
+maman|Oui, dans l'air.
+papa|La cuisine est calme, Amir ?
+enfant-m|Oui, papa.
+narrateur|Deux petits bouts ont suffi.
+narrateur|Un éclat de saladier tient sur le verre.</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2173,6 +2287,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>